<commit_message>
remove spaces from checkv fileds
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99311BF2-83E0-4BF7-9952-B0DE8E57F3E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDEEB2B0-5037-4254-AE17-C53FFBB837D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4931,7 +4931,7 @@
     <t>contig_length_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Contig Length CheckV</t>
+    <t>Contig Length CheckV</t>
   </si>
   <si>
     <t>Length of the sequence as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -4943,7 +4943,7 @@
     <t>provirus_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Provirus CheckV</t>
+    <t>Provirus CheckV</t>
   </si>
   <si>
     <t>Prediction of whether the sequence is a provirus by CheckV v1.1.1 against the default CheckV database v1.5. [Yes/No] For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -4955,7 +4955,7 @@
     <t>proviral_length_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Proviral Length CheckV</t>
+    <t>Proviral Length CheckV</t>
   </si>
   <si>
     <t>If the sequence is predicated as a provirus, the length ofthe provirus, calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -4967,7 +4967,7 @@
     <t>gene_count_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Gene Count CheckV</t>
+    <t>Gene Count CheckV</t>
   </si>
   <si>
     <t>The number of genes in the virus sequence as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -4979,7 +4979,7 @@
     <t>viral_genes_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Viral Genes CheckV</t>
+    <t>Viral Genes CheckV</t>
   </si>
   <si>
     <t>The number of virus genes in the virus sequence as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -4991,7 +4991,7 @@
     <t>host_genes_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Host Genes CheckV</t>
+    <t>Host Genes CheckV</t>
   </si>
   <si>
     <t>The number of host genes as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -5003,7 +5003,7 @@
     <t>quality_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Quality CheckV</t>
+    <t>Quality CheckV</t>
   </si>
   <si>
     <t>Quality tier of the virus genome as noted by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master 
@@ -5021,7 +5021,7 @@
     <t>miuvig_quality_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> MIUVIG Quality CheckV</t>
+    <t>MIUVIG Quality CheckV</t>
   </si>
   <si>
     <t>MIUVIG quality as noted by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -5033,7 +5033,7 @@
     <t>completeness_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Completeness CheckV</t>
+    <t>Completeness CheckV</t>
   </si>
   <si>
     <t>Completeness of the virus genome sequenceas calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -5045,7 +5045,7 @@
     <t>completeness_method_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Completeness Method CheckV</t>
+    <t>Completeness Method CheckV</t>
   </si>
   <si>
     <t>Method of determining the completeness of the virus genome sequence as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -5057,7 +5057,7 @@
     <t>contamination_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Contamination CheckV</t>
+    <t>Contamination CheckV</t>
   </si>
   <si>
     <t>Amount of virus genome sequence contamination as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -5069,7 +5069,7 @@
     <t>kmer_freq_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Kmer Freq CheckV</t>
+    <t>Kmer Freq CheckV</t>
   </si>
   <si>
     <t>Number of times the virus genome was found in the as calculated by CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>
@@ -5081,7 +5081,7 @@
     <t>warnings_checkv</t>
   </si>
   <si>
-    <t xml:space="preserve"> Warnings CheckV</t>
+    <t>Warnings CheckV</t>
   </si>
   <si>
     <t>Warnings generated by running CheckV v1.1.1 against the default CheckV database v1.5. For more information about CheckV please see the tool page at: https://bitbucket.org/berkeleylab/checkv/src/master</t>

</xml_diff>

<commit_message>
Validation field of 0ie has been updated
according to task https://vj.srsoftware.de/task/460/view content of validation field has been append to description and be replaced with valid value.
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95F02E05-0D41-47AE-8ED6-2948F96E31E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{368FE683-6CCE-43A7-B1CE-A2D2BEFB873A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -237,7 +237,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5036" uniqueCount="1804">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5037" uniqueCount="1804">
   <si>
     <t>VJDBv1.1</t>
   </si>
@@ -4843,26 +4843,27 @@
     <t>Coding Strand</t>
   </si>
   <si>
-    <t>True if the current virus sequence is a coding strand. Calculated by part of the ViralClust tool suite. Only intended for ssRNA viruses.</t>
+    <t>True if the current virus sequence is a coding strand. Calculated by part of the ViralClust tool suite. Only intended for ssRNA viruses."TRUE: is coding strand
+FALSE: is reverse complement"</t>
   </si>
   <si>
     <t>TRUE</t>
+  </si>
+  <si>
+    <t>0if</t>
+  </si>
+  <si>
+    <t>host_association_method</t>
+  </si>
+  <si>
+    <t>Host Association Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method by which the fields "Host Accession ID" from NCBI GenBank or "NCBI Taxonomy Lineage" was associated to the virus sequence. Currently (v1.1) either a host association from the data source or PhiSpy prophage prediction. Multiple host associations/predictions separated by semicolons. </t>
   </si>
   <si>
     <t>TRUE: is coding strand
 FALSE: is reverse complement</t>
-  </si>
-  <si>
-    <t>0if</t>
-  </si>
-  <si>
-    <t>host_association_method</t>
-  </si>
-  <si>
-    <t>Host Association Method</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Method by which the fields "Host Accession ID" from NCBI GenBank or "NCBI Taxonomy Lineage" was associated to the virus sequence. Currently (v1.1) either a host association from the data source or PhiSpy prophage prediction. Multiple host associations/predictions separated by semicolons. </t>
   </si>
   <si>
     <t>0ig</t>
@@ -6607,7 +6608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FX237"/>
+  <dimension ref="A1:FX238"/>
   <sheetFormatPr defaultColWidth="23.5703125" defaultRowHeight="25.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24.140625" style="67" bestFit="1" customWidth="1"/>
@@ -44477,7 +44478,7 @@
       <c r="C217" s="54" t="s">
         <v>1519</v>
       </c>
-      <c r="D217" s="75" t="s">
+      <c r="D217" s="71" t="s">
         <v>1520</v>
       </c>
       <c r="E217" s="54" t="s">
@@ -44560,7 +44561,7 @@
         <v>1521</v>
       </c>
       <c r="AV217" s="54" t="s">
-        <v>1522</v>
+        <v>169</v>
       </c>
       <c r="AW217" s="54"/>
       <c r="AX217" s="54"/>
@@ -44570,16 +44571,16 @@
     </row>
     <row r="218" spans="1:53" ht="25.5" customHeight="1">
       <c r="A218" s="64" t="s">
+        <v>1522</v>
+      </c>
+      <c r="B218" s="64" t="s">
         <v>1523</v>
       </c>
-      <c r="B218" s="64" t="s">
+      <c r="C218" s="54" t="s">
         <v>1524</v>
       </c>
-      <c r="C218" s="54" t="s">
+      <c r="D218" s="71" t="s">
         <v>1525</v>
-      </c>
-      <c r="D218" s="71" t="s">
-        <v>1526</v>
       </c>
       <c r="E218" s="54" t="s">
         <v>76</v>
@@ -44660,7 +44661,9 @@
       <c r="AS218" s="54"/>
       <c r="AT218" s="54"/>
       <c r="AU218" s="55"/>
-      <c r="AV218" s="54"/>
+      <c r="AV218" s="54" t="s">
+        <v>1526</v>
+      </c>
       <c r="AW218" s="54"/>
       <c r="AX218" s="54"/>
       <c r="AY218" s="54"/>
@@ -45249,7 +45252,7 @@
       <c r="AZ224" s="54"/>
       <c r="BA224" s="54"/>
     </row>
-    <row r="225" spans="1:53" ht="25.5" customHeight="1">
+    <row r="225" spans="1:180" ht="25.5" customHeight="1">
       <c r="A225" s="64" t="s">
         <v>1551</v>
       </c>
@@ -45344,7 +45347,7 @@
       <c r="AZ225" s="54"/>
       <c r="BA225" s="54"/>
     </row>
-    <row r="226" spans="1:53" ht="25.5" customHeight="1">
+    <row r="226" spans="1:180" ht="25.5" customHeight="1">
       <c r="A226" s="64" t="s">
         <v>1555</v>
       </c>
@@ -45439,7 +45442,7 @@
       <c r="AZ226" s="54"/>
       <c r="BA226" s="54"/>
     </row>
-    <row r="227" spans="1:53" ht="25.5" customHeight="1">
+    <row r="227" spans="1:180" ht="25.5" customHeight="1">
       <c r="A227" s="64" t="s">
         <v>1559</v>
       </c>
@@ -45534,7 +45537,7 @@
       <c r="AZ227" s="54"/>
       <c r="BA227" s="54"/>
     </row>
-    <row r="228" spans="1:53" ht="25.5" customHeight="1">
+    <row r="228" spans="1:180" ht="25.5" customHeight="1">
       <c r="A228" s="64" t="s">
         <v>1563</v>
       </c>
@@ -45629,7 +45632,7 @@
       <c r="AZ228" s="54"/>
       <c r="BA228" s="54"/>
     </row>
-    <row r="229" spans="1:53" ht="25.5" customHeight="1">
+    <row r="229" spans="1:180" ht="25.5" customHeight="1">
       <c r="A229" s="64" t="s">
         <v>1567</v>
       </c>
@@ -45724,7 +45727,7 @@
       <c r="AZ229" s="54"/>
       <c r="BA229" s="54"/>
     </row>
-    <row r="230" spans="1:53" ht="25.5" customHeight="1">
+    <row r="230" spans="1:180" ht="25.5" customHeight="1">
       <c r="A230" s="64" t="s">
         <v>1571</v>
       </c>
@@ -45819,7 +45822,7 @@
       <c r="AZ230" s="54"/>
       <c r="BA230" s="54"/>
     </row>
-    <row r="231" spans="1:53" ht="25.5" customHeight="1">
+    <row r="231" spans="1:180" ht="25.5" customHeight="1">
       <c r="A231" s="64" t="s">
         <v>1575</v>
       </c>
@@ -45914,7 +45917,7 @@
       <c r="AZ231" s="54"/>
       <c r="BA231" s="54"/>
     </row>
-    <row r="232" spans="1:53" ht="25.5" customHeight="1">
+    <row r="232" spans="1:180" ht="25.5" customHeight="1">
       <c r="A232" s="64" t="s">
         <v>1579</v>
       </c>
@@ -46009,7 +46012,7 @@
       <c r="AZ232" s="54"/>
       <c r="BA232" s="54"/>
     </row>
-    <row r="233" spans="1:53" ht="25.5" customHeight="1">
+    <row r="233" spans="1:180" ht="25.5" customHeight="1">
       <c r="A233" s="64" t="s">
         <v>1583</v>
       </c>
@@ -46104,7 +46107,7 @@
       <c r="AZ233" s="54"/>
       <c r="BA233" s="54"/>
     </row>
-    <row r="234" spans="1:53" ht="25.5" customHeight="1">
+    <row r="234" spans="1:180" ht="25.5" customHeight="1">
       <c r="A234" s="64" t="s">
         <v>1587</v>
       </c>
@@ -46199,7 +46202,7 @@
       <c r="AZ234" s="54"/>
       <c r="BA234" s="54"/>
     </row>
-    <row r="235" spans="1:53" ht="25.5" customHeight="1">
+    <row r="235" spans="1:180" ht="25.5" customHeight="1">
       <c r="A235" s="64" t="s">
         <v>1591</v>
       </c>
@@ -46294,7 +46297,7 @@
       <c r="AZ235" s="54"/>
       <c r="BA235" s="54"/>
     </row>
-    <row r="236" spans="1:53" ht="25.5" customHeight="1">
+    <row r="236" spans="1:180" ht="25.5" customHeight="1">
       <c r="A236" s="64" t="s">
         <v>1595</v>
       </c>
@@ -46389,7 +46392,7 @@
       <c r="AZ236" s="54"/>
       <c r="BA236" s="54"/>
     </row>
-    <row r="237" spans="1:53" ht="25.5" customHeight="1">
+    <row r="237" spans="1:180" ht="25.5" customHeight="1">
       <c r="A237" s="64" t="s">
         <v>1599</v>
       </c>
@@ -46486,14 +46489,196 @@
         <v>1602</v>
       </c>
     </row>
+    <row r="238" spans="1:180" ht="25.5" customHeight="1">
+      <c r="A238" s="64"/>
+      <c r="B238" s="64"/>
+      <c r="C238" s="64"/>
+      <c r="D238" s="64"/>
+      <c r="E238" s="64"/>
+      <c r="F238" s="64"/>
+      <c r="G238" s="64"/>
+      <c r="H238" s="64"/>
+      <c r="I238" s="64"/>
+      <c r="J238" s="64"/>
+      <c r="K238" s="64"/>
+      <c r="L238" s="64"/>
+      <c r="M238" s="64"/>
+      <c r="N238" s="64"/>
+      <c r="O238" s="64"/>
+      <c r="P238" s="64"/>
+      <c r="Q238" s="64"/>
+      <c r="R238" s="64"/>
+      <c r="S238" s="64"/>
+      <c r="T238" s="64"/>
+      <c r="U238" s="64"/>
+      <c r="V238" s="64"/>
+      <c r="W238" s="64"/>
+      <c r="X238" s="64"/>
+      <c r="Y238" s="64"/>
+      <c r="Z238" s="64"/>
+      <c r="AA238" s="64"/>
+      <c r="AB238" s="64"/>
+      <c r="AC238" s="64"/>
+      <c r="AD238" s="64"/>
+      <c r="AE238" s="64"/>
+      <c r="AF238" s="64"/>
+      <c r="AG238" s="64"/>
+      <c r="AH238" s="64"/>
+      <c r="AI238" s="64"/>
+      <c r="AJ238" s="64"/>
+      <c r="AK238" s="64"/>
+      <c r="AL238" s="64"/>
+      <c r="AM238" s="64"/>
+      <c r="AN238" s="64"/>
+      <c r="AO238" s="64"/>
+      <c r="AP238" s="64"/>
+      <c r="AQ238" s="64"/>
+      <c r="AR238" s="64"/>
+      <c r="AS238" s="64"/>
+      <c r="AT238" s="64"/>
+      <c r="AU238" s="64"/>
+      <c r="AV238" s="64"/>
+      <c r="AW238" s="64"/>
+      <c r="AX238" s="64"/>
+      <c r="AY238" s="64"/>
+      <c r="AZ238" s="64"/>
+      <c r="BA238" s="64"/>
+      <c r="BB238" s="64"/>
+      <c r="BC238" s="64"/>
+      <c r="BD238" s="64"/>
+      <c r="BE238" s="64"/>
+      <c r="BF238" s="64"/>
+      <c r="BG238" s="64"/>
+      <c r="BH238" s="64"/>
+      <c r="BI238" s="64"/>
+      <c r="BJ238" s="64"/>
+      <c r="BK238" s="64"/>
+      <c r="BL238" s="64"/>
+      <c r="BM238" s="64"/>
+      <c r="BN238" s="64"/>
+      <c r="BO238" s="64"/>
+      <c r="BP238" s="64"/>
+      <c r="BQ238" s="64"/>
+      <c r="BR238" s="64"/>
+      <c r="BS238" s="64"/>
+      <c r="BT238" s="64"/>
+      <c r="BU238" s="64"/>
+      <c r="BV238" s="64"/>
+      <c r="BW238" s="64"/>
+      <c r="BX238" s="64"/>
+      <c r="BY238" s="64"/>
+      <c r="BZ238" s="64"/>
+      <c r="CA238" s="64"/>
+      <c r="CB238" s="64"/>
+      <c r="CC238" s="64"/>
+      <c r="CD238" s="64"/>
+      <c r="CE238" s="64"/>
+      <c r="CF238" s="64"/>
+      <c r="CG238" s="64"/>
+      <c r="CH238" s="64"/>
+      <c r="CI238" s="64"/>
+      <c r="CJ238" s="64"/>
+      <c r="CK238" s="64"/>
+      <c r="CL238" s="64"/>
+      <c r="CM238" s="64"/>
+      <c r="CN238" s="64"/>
+      <c r="CO238" s="64"/>
+      <c r="CP238" s="64"/>
+      <c r="CQ238" s="64"/>
+      <c r="CR238" s="64"/>
+      <c r="CS238" s="64"/>
+      <c r="CT238" s="64"/>
+      <c r="CU238" s="64"/>
+      <c r="CV238" s="64"/>
+      <c r="CW238" s="64"/>
+      <c r="CX238" s="64"/>
+      <c r="CY238" s="64"/>
+      <c r="CZ238" s="64"/>
+      <c r="DA238" s="64"/>
+      <c r="DB238" s="64"/>
+      <c r="DC238" s="64"/>
+      <c r="DD238" s="64"/>
+      <c r="DE238" s="64"/>
+      <c r="DF238" s="64"/>
+      <c r="DG238" s="64"/>
+      <c r="DH238" s="64"/>
+      <c r="DI238" s="64"/>
+      <c r="DJ238" s="64"/>
+      <c r="DK238" s="64"/>
+      <c r="DL238" s="64"/>
+      <c r="DM238" s="64"/>
+      <c r="DN238" s="64"/>
+      <c r="DO238" s="64"/>
+      <c r="DP238" s="64"/>
+      <c r="DQ238" s="64"/>
+      <c r="DR238" s="64"/>
+      <c r="DS238" s="64"/>
+      <c r="DT238" s="64"/>
+      <c r="DU238" s="64"/>
+      <c r="DV238" s="64"/>
+      <c r="DW238" s="64"/>
+      <c r="DX238" s="64"/>
+      <c r="DY238" s="64"/>
+      <c r="DZ238" s="64"/>
+      <c r="EA238" s="64"/>
+      <c r="EB238" s="64"/>
+      <c r="EC238" s="64"/>
+      <c r="ED238" s="64"/>
+      <c r="EE238" s="64"/>
+      <c r="EF238" s="64"/>
+      <c r="EG238" s="64"/>
+      <c r="EH238" s="64"/>
+      <c r="EI238" s="64"/>
+      <c r="EJ238" s="64"/>
+      <c r="EK238" s="64"/>
+      <c r="EL238" s="64"/>
+      <c r="EM238" s="64"/>
+      <c r="EN238" s="64"/>
+      <c r="EO238" s="64"/>
+      <c r="EP238" s="64"/>
+      <c r="EQ238" s="64"/>
+      <c r="ER238" s="64"/>
+      <c r="ES238" s="64"/>
+      <c r="ET238" s="64"/>
+      <c r="EU238" s="64"/>
+      <c r="EV238" s="64"/>
+      <c r="EW238" s="64"/>
+      <c r="EX238" s="64"/>
+      <c r="EY238" s="64"/>
+      <c r="EZ238" s="64"/>
+      <c r="FA238" s="64"/>
+      <c r="FB238" s="64"/>
+      <c r="FC238" s="64"/>
+      <c r="FD238" s="64"/>
+      <c r="FE238" s="64"/>
+      <c r="FF238" s="64"/>
+      <c r="FG238" s="64"/>
+      <c r="FH238" s="64"/>
+      <c r="FI238" s="64"/>
+      <c r="FJ238" s="64"/>
+      <c r="FK238" s="64"/>
+      <c r="FL238" s="64"/>
+      <c r="FM238" s="64"/>
+      <c r="FN238" s="64"/>
+      <c r="FO238" s="64"/>
+      <c r="FP238" s="64"/>
+      <c r="FQ238" s="64"/>
+      <c r="FR238" s="64"/>
+      <c r="FS238" s="64"/>
+      <c r="FT238" s="64"/>
+      <c r="FU238" s="64"/>
+      <c r="FV238" s="64"/>
+      <c r="FW238" s="64"/>
+      <c r="FX238" s="64"/>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:BC237">
     <sortCondition ref="A5:A237"/>
   </sortState>
-  <conditionalFormatting sqref="A8:B1048576 A5:A7 A1 A2:B4 C3:BC3">
+  <conditionalFormatting sqref="A8:B237 A5:A7 A1 A2:B4 C3:BC3 A239:B1048576 A238:FX238">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E2 E4:E1048576">
+  <conditionalFormatting sqref="E1:E2 E4:E237 E239:E1048576">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"boolean"</formula>
     </cfRule>

</xml_diff>